<commit_message>
Update CRM Journeys workbook and add Fibre/Postpaid BRSD diagram outputs
Refresh CRM_Journeys_Final_Updated_with_Type.xlsx, and add the
vfq-diagram-engine gap-analysis deliverables for the Fibre BRSD (vs.
implementation and vs. swimlane) plus process notes for the Mobile
Postpaid Activation BRSD.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Journeys/CRM_Journeys_Final_Updated_with_Type.xlsx
+++ b/Journeys/CRM_Journeys_Final_Updated_with_Type.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/parithimalsaravanan/claude-projects/vfq/Journeys/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C5B3CA4-27DB-644C-98F5-9B94E30F6AAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C639CBF9-47C6-9240-8B69-0C453CF6FB23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1534,7 +1534,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:L166"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1697,7 +1696,7 @@
       </c>
       <c r="L4" s="11"/>
     </row>
-    <row r="5" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="10">
         <v>4</v>
       </c>
@@ -2057,7 +2056,7 @@
       </c>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A15" s="10">
         <v>14</v>
       </c>
@@ -2129,7 +2128,7 @@
       </c>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A17" s="10">
         <v>16</v>
       </c>
@@ -2165,7 +2164,7 @@
       </c>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="10">
         <v>17</v>
       </c>
@@ -2201,7 +2200,7 @@
       </c>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="10">
         <v>18</v>
       </c>
@@ -2237,7 +2236,7 @@
       </c>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="1:12" ht="48" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12" ht="48" x14ac:dyDescent="0.2">
       <c r="A20" s="10">
         <v>19</v>
       </c>
@@ -2273,7 +2272,7 @@
       </c>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="10">
         <v>20</v>
       </c>
@@ -2309,7 +2308,7 @@
       </c>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="1:12" ht="48" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" ht="48" x14ac:dyDescent="0.2">
       <c r="A22" s="10">
         <v>21</v>
       </c>
@@ -2345,7 +2344,7 @@
       </c>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="10">
         <v>22</v>
       </c>
@@ -2381,7 +2380,7 @@
       </c>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A24" s="10">
         <v>23</v>
       </c>
@@ -2417,7 +2416,7 @@
       </c>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A25" s="10">
         <v>24</v>
       </c>
@@ -2453,7 +2452,7 @@
       </c>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="10">
         <v>25</v>
       </c>
@@ -2561,7 +2560,7 @@
       </c>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="10">
         <v>28</v>
       </c>
@@ -2597,7 +2596,7 @@
       </c>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A30" s="10">
         <v>29</v>
       </c>
@@ -2633,7 +2632,7 @@
       </c>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="10">
         <v>30</v>
       </c>
@@ -2669,7 +2668,7 @@
       </c>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A32" s="10">
         <v>31</v>
       </c>
@@ -2707,7 +2706,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="10">
         <v>32</v>
       </c>
@@ -2743,7 +2742,7 @@
       </c>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="10">
         <v>33</v>
       </c>
@@ -2779,7 +2778,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="10">
         <v>34</v>
       </c>
@@ -2815,7 +2814,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="10">
         <v>35</v>
       </c>
@@ -2851,7 +2850,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="10">
         <v>36</v>
       </c>
@@ -2923,7 +2922,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="10">
         <v>38</v>
       </c>
@@ -2959,7 +2958,7 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="10">
         <v>39</v>
       </c>
@@ -2995,7 +2994,7 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="10">
         <v>40</v>
       </c>
@@ -3031,7 +3030,7 @@
       </c>
       <c r="L41" s="11"/>
     </row>
-    <row r="42" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="10">
         <v>41</v>
       </c>
@@ -3067,7 +3066,7 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="10">
         <v>42</v>
       </c>
@@ -3103,7 +3102,7 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A44" s="10">
         <v>43</v>
       </c>
@@ -3141,7 +3140,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="45" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="10">
         <v>44</v>
       </c>
@@ -3177,7 +3176,7 @@
       </c>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="10">
         <v>45</v>
       </c>
@@ -3215,7 +3214,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="47" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="10">
         <v>46</v>
       </c>
@@ -3253,7 +3252,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="48" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" s="10">
         <v>47</v>
       </c>
@@ -3291,7 +3290,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="49" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" s="10">
         <v>48</v>
       </c>
@@ -3327,7 +3326,7 @@
       </c>
       <c r="L49" s="11"/>
     </row>
-    <row r="50" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" s="10">
         <v>49</v>
       </c>
@@ -3363,7 +3362,7 @@
       </c>
       <c r="L50" s="11"/>
     </row>
-    <row r="51" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A51" s="10">
         <v>50</v>
       </c>
@@ -3401,7 +3400,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="52" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="10">
         <v>51</v>
       </c>
@@ -3437,7 +3436,7 @@
       </c>
       <c r="L52" s="11"/>
     </row>
-    <row r="53" spans="1:12" ht="48" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:12" ht="48" x14ac:dyDescent="0.2">
       <c r="A53" s="10">
         <v>52</v>
       </c>
@@ -3473,7 +3472,7 @@
       </c>
       <c r="L53" s="11"/>
     </row>
-    <row r="54" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" s="10">
         <v>53</v>
       </c>
@@ -3509,7 +3508,7 @@
       </c>
       <c r="L54" s="11"/>
     </row>
-    <row r="55" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" s="10">
         <v>54</v>
       </c>
@@ -3545,7 +3544,7 @@
       </c>
       <c r="L55" s="11"/>
     </row>
-    <row r="56" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="10">
         <v>55</v>
       </c>
@@ -3581,7 +3580,7 @@
       </c>
       <c r="L56" s="11"/>
     </row>
-    <row r="57" spans="1:12" ht="48" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:12" ht="48" x14ac:dyDescent="0.2">
       <c r="A57" s="10">
         <v>56</v>
       </c>
@@ -3617,7 +3616,7 @@
       </c>
       <c r="L57" s="11"/>
     </row>
-    <row r="58" spans="1:12" ht="48" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:12" ht="48" x14ac:dyDescent="0.2">
       <c r="A58" s="10">
         <v>57</v>
       </c>
@@ -3653,7 +3652,7 @@
       </c>
       <c r="L58" s="11"/>
     </row>
-    <row r="59" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A59" s="10">
         <v>58</v>
       </c>
@@ -3689,7 +3688,7 @@
       </c>
       <c r="L59" s="11"/>
     </row>
-    <row r="60" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A60" s="10">
         <v>59</v>
       </c>
@@ -3725,7 +3724,7 @@
       </c>
       <c r="L60" s="11"/>
     </row>
-    <row r="61" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" s="10">
         <v>60</v>
       </c>
@@ -3761,7 +3760,7 @@
       </c>
       <c r="L61" s="11"/>
     </row>
-    <row r="62" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" s="10">
         <v>61</v>
       </c>
@@ -3797,7 +3796,7 @@
       </c>
       <c r="L62" s="11"/>
     </row>
-    <row r="63" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A63" s="10">
         <v>62</v>
       </c>
@@ -3833,7 +3832,7 @@
       </c>
       <c r="L63" s="11"/>
     </row>
-    <row r="64" spans="1:12" ht="48" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:12" ht="48" x14ac:dyDescent="0.2">
       <c r="A64" s="10">
         <v>63</v>
       </c>
@@ -3869,7 +3868,7 @@
       </c>
       <c r="L64" s="11"/>
     </row>
-    <row r="65" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A65" s="10">
         <v>64</v>
       </c>
@@ -3905,7 +3904,7 @@
       </c>
       <c r="L65" s="11"/>
     </row>
-    <row r="66" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="10">
         <v>65</v>
       </c>
@@ -3941,7 +3940,7 @@
       </c>
       <c r="L66" s="11"/>
     </row>
-    <row r="67" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A67" s="10">
         <v>66</v>
       </c>
@@ -3977,7 +3976,7 @@
       </c>
       <c r="L67" s="11"/>
     </row>
-    <row r="68" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A68" s="10">
         <v>67</v>
       </c>
@@ -4013,7 +4012,7 @@
       </c>
       <c r="L68" s="11"/>
     </row>
-    <row r="69" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A69" s="10">
         <v>68</v>
       </c>
@@ -4049,7 +4048,7 @@
       </c>
       <c r="L69" s="11"/>
     </row>
-    <row r="70" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A70" s="10">
         <v>69</v>
       </c>
@@ -4085,7 +4084,7 @@
       </c>
       <c r="L70" s="11"/>
     </row>
-    <row r="71" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A71" s="10">
         <v>70</v>
       </c>
@@ -4157,7 +4156,7 @@
       </c>
       <c r="L72" s="11"/>
     </row>
-    <row r="73" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A73" s="10">
         <v>72</v>
       </c>
@@ -4193,7 +4192,7 @@
       </c>
       <c r="L73" s="11"/>
     </row>
-    <row r="74" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A74" s="10">
         <v>73</v>
       </c>
@@ -4229,7 +4228,7 @@
       </c>
       <c r="L74" s="11"/>
     </row>
-    <row r="75" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A75" s="10">
         <v>74</v>
       </c>
@@ -4265,7 +4264,7 @@
       </c>
       <c r="L75" s="11"/>
     </row>
-    <row r="76" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A76" s="10">
         <v>75</v>
       </c>
@@ -4301,7 +4300,7 @@
       </c>
       <c r="L76" s="11"/>
     </row>
-    <row r="77" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A77" s="10">
         <v>76</v>
       </c>
@@ -4337,7 +4336,7 @@
       </c>
       <c r="L77" s="11"/>
     </row>
-    <row r="78" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A78" s="10">
         <v>77</v>
       </c>
@@ -4373,7 +4372,7 @@
       </c>
       <c r="L78" s="11"/>
     </row>
-    <row r="79" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A79" s="10">
         <v>78</v>
       </c>
@@ -4409,7 +4408,7 @@
       </c>
       <c r="L79" s="11"/>
     </row>
-    <row r="80" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A80" s="10">
         <v>79</v>
       </c>
@@ -4445,7 +4444,7 @@
       </c>
       <c r="L80" s="11"/>
     </row>
-    <row r="81" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A81" s="10">
         <v>80</v>
       </c>
@@ -4481,7 +4480,7 @@
       </c>
       <c r="L81" s="11"/>
     </row>
-    <row r="82" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A82" s="10">
         <v>81</v>
       </c>
@@ -4517,7 +4516,7 @@
       </c>
       <c r="L82" s="11"/>
     </row>
-    <row r="83" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A83" s="10">
         <v>82</v>
       </c>
@@ -4553,7 +4552,7 @@
       </c>
       <c r="L83" s="11"/>
     </row>
-    <row r="84" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A84" s="10">
         <v>83</v>
       </c>
@@ -4589,7 +4588,7 @@
       </c>
       <c r="L84" s="11"/>
     </row>
-    <row r="85" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A85" s="10">
         <v>84</v>
       </c>
@@ -4625,7 +4624,7 @@
       </c>
       <c r="L85" s="11"/>
     </row>
-    <row r="86" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A86" s="10">
         <v>85</v>
       </c>
@@ -4661,7 +4660,7 @@
       </c>
       <c r="L86" s="11"/>
     </row>
-    <row r="87" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A87" s="10">
         <v>86</v>
       </c>
@@ -4697,7 +4696,7 @@
       </c>
       <c r="L87" s="11"/>
     </row>
-    <row r="88" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A88" s="10">
         <v>87</v>
       </c>
@@ -4733,7 +4732,7 @@
       </c>
       <c r="L88" s="11"/>
     </row>
-    <row r="89" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A89" s="10">
         <v>88</v>
       </c>
@@ -4769,7 +4768,7 @@
       </c>
       <c r="L89" s="11"/>
     </row>
-    <row r="90" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A90" s="10">
         <v>89</v>
       </c>
@@ -4805,7 +4804,7 @@
       </c>
       <c r="L90" s="11"/>
     </row>
-    <row r="91" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A91" s="10">
         <v>90</v>
       </c>
@@ -4841,7 +4840,7 @@
       </c>
       <c r="L91" s="11"/>
     </row>
-    <row r="92" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A92" s="10">
         <v>91</v>
       </c>
@@ -4877,7 +4876,7 @@
       </c>
       <c r="L92" s="11"/>
     </row>
-    <row r="93" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A93" s="10">
         <v>92</v>
       </c>
@@ -4913,7 +4912,7 @@
       </c>
       <c r="L93" s="11"/>
     </row>
-    <row r="94" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A94" s="10">
         <v>93</v>
       </c>
@@ -4949,7 +4948,7 @@
       </c>
       <c r="L94" s="11"/>
     </row>
-    <row r="95" spans="1:12" ht="80" hidden="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:12" ht="80" x14ac:dyDescent="0.2">
       <c r="A95" s="10">
         <v>94</v>
       </c>
@@ -4985,7 +4984,7 @@
       </c>
       <c r="L95" s="11"/>
     </row>
-    <row r="96" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A96" s="10">
         <v>95</v>
       </c>
@@ -5021,7 +5020,7 @@
       </c>
       <c r="L96" s="11"/>
     </row>
-    <row r="97" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A97" s="10">
         <v>96</v>
       </c>
@@ -5057,7 +5056,7 @@
       </c>
       <c r="L97" s="11"/>
     </row>
-    <row r="98" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A98" s="10">
         <v>97</v>
       </c>
@@ -5093,7 +5092,7 @@
       </c>
       <c r="L98" s="11"/>
     </row>
-    <row r="99" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A99" s="10">
         <v>98</v>
       </c>
@@ -5129,7 +5128,7 @@
       </c>
       <c r="L99" s="11"/>
     </row>
-    <row r="100" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A100" s="10">
         <v>99</v>
       </c>
@@ -5165,7 +5164,7 @@
       </c>
       <c r="L100" s="11"/>
     </row>
-    <row r="101" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A101" s="10">
         <v>100</v>
       </c>
@@ -5201,7 +5200,7 @@
       </c>
       <c r="L101" s="11"/>
     </row>
-    <row r="102" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A102" s="10">
         <v>101</v>
       </c>
@@ -5237,7 +5236,7 @@
       </c>
       <c r="L102" s="11"/>
     </row>
-    <row r="103" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A103" s="10">
         <v>102</v>
       </c>
@@ -5273,7 +5272,7 @@
       </c>
       <c r="L103" s="11"/>
     </row>
-    <row r="104" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A104" s="10">
         <v>103</v>
       </c>
@@ -5309,7 +5308,7 @@
       </c>
       <c r="L104" s="11"/>
     </row>
-    <row r="105" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A105" s="10">
         <v>104</v>
       </c>
@@ -5345,7 +5344,7 @@
       </c>
       <c r="L105" s="11"/>
     </row>
-    <row r="106" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A106" s="10">
         <v>105</v>
       </c>
@@ -5381,7 +5380,7 @@
       </c>
       <c r="L106" s="11"/>
     </row>
-    <row r="107" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A107" s="10">
         <v>106</v>
       </c>
@@ -5417,7 +5416,7 @@
       </c>
       <c r="L107" s="11"/>
     </row>
-    <row r="108" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A108" s="10">
         <v>107</v>
       </c>
@@ -5453,7 +5452,7 @@
       </c>
       <c r="L108" s="11"/>
     </row>
-    <row r="109" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A109" s="10">
         <v>108</v>
       </c>
@@ -5489,7 +5488,7 @@
       </c>
       <c r="L109" s="11"/>
     </row>
-    <row r="110" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A110" s="10">
         <v>109</v>
       </c>
@@ -5525,7 +5524,7 @@
       </c>
       <c r="L110" s="11"/>
     </row>
-    <row r="111" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A111" s="10">
         <v>110</v>
       </c>
@@ -5561,7 +5560,7 @@
       </c>
       <c r="L111" s="11"/>
     </row>
-    <row r="112" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A112" s="10">
         <v>111</v>
       </c>
@@ -5597,7 +5596,7 @@
       </c>
       <c r="L112" s="11"/>
     </row>
-    <row r="113" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A113" s="10">
         <v>112</v>
       </c>
@@ -5633,7 +5632,7 @@
       </c>
       <c r="L113" s="11"/>
     </row>
-    <row r="114" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A114" s="10">
         <v>113</v>
       </c>
@@ -5669,7 +5668,7 @@
       </c>
       <c r="L114" s="11"/>
     </row>
-    <row r="115" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A115" s="10">
         <v>114</v>
       </c>
@@ -5705,7 +5704,7 @@
       </c>
       <c r="L115" s="11"/>
     </row>
-    <row r="116" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A116" s="10">
         <v>115</v>
       </c>
@@ -5741,7 +5740,7 @@
       </c>
       <c r="L116" s="11"/>
     </row>
-    <row r="117" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A117" s="10">
         <v>116</v>
       </c>
@@ -5777,7 +5776,7 @@
       </c>
       <c r="L117" s="11"/>
     </row>
-    <row r="118" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A118" s="10">
         <v>117</v>
       </c>
@@ -5813,7 +5812,7 @@
       </c>
       <c r="L118" s="11"/>
     </row>
-    <row r="119" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A119" s="10">
         <v>118</v>
       </c>
@@ -5849,7 +5848,7 @@
       </c>
       <c r="L119" s="11"/>
     </row>
-    <row r="120" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A120" s="10">
         <v>119</v>
       </c>
@@ -5885,7 +5884,7 @@
       </c>
       <c r="L120" s="11"/>
     </row>
-    <row r="121" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A121" s="10">
         <v>120</v>
       </c>
@@ -5921,7 +5920,7 @@
       </c>
       <c r="L121" s="11"/>
     </row>
-    <row r="122" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A122" s="10">
         <v>121</v>
       </c>
@@ -5957,7 +5956,7 @@
       </c>
       <c r="L122" s="11"/>
     </row>
-    <row r="123" spans="1:12" ht="48" hidden="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:12" ht="48" x14ac:dyDescent="0.2">
       <c r="A123" s="10">
         <v>122</v>
       </c>
@@ -5993,7 +5992,7 @@
       </c>
       <c r="L123" s="11"/>
     </row>
-    <row r="124" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A124" s="10">
         <v>123</v>
       </c>
@@ -6029,7 +6028,7 @@
       </c>
       <c r="L124" s="11"/>
     </row>
-    <row r="125" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A125" s="10">
         <v>124</v>
       </c>
@@ -6065,7 +6064,7 @@
       </c>
       <c r="L125" s="11"/>
     </row>
-    <row r="126" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A126" s="10">
         <v>125</v>
       </c>
@@ -6101,7 +6100,7 @@
       </c>
       <c r="L126" s="11"/>
     </row>
-    <row r="127" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A127" s="10">
         <v>126</v>
       </c>
@@ -6137,7 +6136,7 @@
       </c>
       <c r="L127" s="11"/>
     </row>
-    <row r="128" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A128" s="10">
         <v>127</v>
       </c>
@@ -6173,7 +6172,7 @@
       </c>
       <c r="L128" s="11"/>
     </row>
-    <row r="129" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A129" s="10">
         <v>128</v>
       </c>
@@ -6209,7 +6208,7 @@
       </c>
       <c r="L129" s="11"/>
     </row>
-    <row r="130" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A130" s="10">
         <v>129</v>
       </c>
@@ -6245,7 +6244,7 @@
       </c>
       <c r="L130" s="11"/>
     </row>
-    <row r="131" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A131" s="10">
         <v>130</v>
       </c>
@@ -6281,7 +6280,7 @@
       </c>
       <c r="L131" s="11"/>
     </row>
-    <row r="132" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A132" s="10">
         <v>131</v>
       </c>
@@ -6317,7 +6316,7 @@
       </c>
       <c r="L132" s="11"/>
     </row>
-    <row r="133" spans="1:12" ht="80" hidden="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:12" ht="80" x14ac:dyDescent="0.2">
       <c r="A133" s="10">
         <v>132</v>
       </c>
@@ -6353,7 +6352,7 @@
       </c>
       <c r="L133" s="11"/>
     </row>
-    <row r="134" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A134" s="10">
         <v>133</v>
       </c>
@@ -6389,7 +6388,7 @@
       </c>
       <c r="L134" s="11"/>
     </row>
-    <row r="135" spans="1:12" ht="48" hidden="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:12" ht="48" x14ac:dyDescent="0.2">
       <c r="A135" s="10">
         <v>134</v>
       </c>
@@ -6425,7 +6424,7 @@
       </c>
       <c r="L135" s="11"/>
     </row>
-    <row r="136" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A136" s="10">
         <v>135</v>
       </c>
@@ -6461,7 +6460,7 @@
       </c>
       <c r="L136" s="11"/>
     </row>
-    <row r="137" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A137" s="10">
         <v>136</v>
       </c>
@@ -6497,7 +6496,7 @@
       </c>
       <c r="L137" s="11"/>
     </row>
-    <row r="138" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A138" s="10">
         <v>137</v>
       </c>
@@ -6533,7 +6532,7 @@
       </c>
       <c r="L138" s="11"/>
     </row>
-    <row r="139" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A139" s="10">
         <v>138</v>
       </c>
@@ -6569,7 +6568,7 @@
       </c>
       <c r="L139" s="11"/>
     </row>
-    <row r="140" spans="1:12" ht="48" hidden="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:12" ht="48" x14ac:dyDescent="0.2">
       <c r="A140" s="10">
         <v>139</v>
       </c>
@@ -6605,7 +6604,7 @@
       </c>
       <c r="L140" s="11"/>
     </row>
-    <row r="141" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A141" s="10">
         <v>140</v>
       </c>
@@ -6641,7 +6640,7 @@
       </c>
       <c r="L141" s="11"/>
     </row>
-    <row r="142" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A142" s="10">
         <v>141</v>
       </c>
@@ -6677,7 +6676,7 @@
       </c>
       <c r="L142" s="11"/>
     </row>
-    <row r="143" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A143" s="10">
         <v>142</v>
       </c>
@@ -6713,7 +6712,7 @@
       </c>
       <c r="L143" s="11"/>
     </row>
-    <row r="144" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A144" s="10">
         <v>143</v>
       </c>
@@ -6749,7 +6748,7 @@
       </c>
       <c r="L144" s="11"/>
     </row>
-    <row r="145" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A145" s="10">
         <v>144</v>
       </c>
@@ -6785,7 +6784,7 @@
       </c>
       <c r="L145" s="11"/>
     </row>
-    <row r="146" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A146" s="10">
         <v>145</v>
       </c>
@@ -6821,7 +6820,7 @@
       </c>
       <c r="L146" s="11"/>
     </row>
-    <row r="147" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A147" s="10">
         <v>146</v>
       </c>
@@ -6857,7 +6856,7 @@
       </c>
       <c r="L147" s="11"/>
     </row>
-    <row r="148" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A148" s="10">
         <v>147</v>
       </c>
@@ -6893,7 +6892,7 @@
       </c>
       <c r="L148" s="11"/>
     </row>
-    <row r="149" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A149" s="10">
         <v>148</v>
       </c>
@@ -6929,7 +6928,7 @@
       </c>
       <c r="L149" s="11"/>
     </row>
-    <row r="150" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A150" s="10">
         <v>149</v>
       </c>
@@ -6965,7 +6964,7 @@
       </c>
       <c r="L150" s="11"/>
     </row>
-    <row r="151" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A151" s="10">
         <v>150</v>
       </c>
@@ -7001,7 +7000,7 @@
       </c>
       <c r="L151" s="11"/>
     </row>
-    <row r="152" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A152" s="10">
         <v>151</v>
       </c>
@@ -7037,7 +7036,7 @@
       </c>
       <c r="L152" s="11"/>
     </row>
-    <row r="153" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A153" s="10">
         <v>152</v>
       </c>
@@ -7073,7 +7072,7 @@
       </c>
       <c r="L153" s="11"/>
     </row>
-    <row r="154" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A154" s="10">
         <v>153</v>
       </c>
@@ -7109,7 +7108,7 @@
       </c>
       <c r="L154" s="11"/>
     </row>
-    <row r="155" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A155" s="10">
         <v>154</v>
       </c>
@@ -7145,7 +7144,7 @@
       </c>
       <c r="L155" s="11"/>
     </row>
-    <row r="156" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A156" s="10">
         <v>155</v>
       </c>
@@ -7181,7 +7180,7 @@
       </c>
       <c r="L156" s="11"/>
     </row>
-    <row r="157" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A157" s="10">
         <v>156</v>
       </c>
@@ -7217,7 +7216,7 @@
       </c>
       <c r="L157" s="11"/>
     </row>
-    <row r="158" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A158" s="10">
         <v>157</v>
       </c>
@@ -7253,7 +7252,7 @@
       </c>
       <c r="L158" s="11"/>
     </row>
-    <row r="159" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A159" s="10">
         <v>158</v>
       </c>
@@ -7289,7 +7288,7 @@
       </c>
       <c r="L159" s="11"/>
     </row>
-    <row r="160" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A160" s="10">
         <v>159</v>
       </c>
@@ -7325,7 +7324,7 @@
       </c>
       <c r="L160" s="11"/>
     </row>
-    <row r="161" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A161" s="10">
         <v>160</v>
       </c>
@@ -7361,7 +7360,7 @@
       </c>
       <c r="L161" s="11"/>
     </row>
-    <row r="162" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A162" s="10">
         <v>161</v>
       </c>
@@ -7397,7 +7396,7 @@
       </c>
       <c r="L162" s="11"/>
     </row>
-    <row r="163" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A163" s="10">
         <v>162</v>
       </c>
@@ -7433,7 +7432,7 @@
       </c>
       <c r="L163" s="11"/>
     </row>
-    <row r="164" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A164" s="10">
         <v>163</v>
       </c>
@@ -7469,7 +7468,7 @@
       </c>
       <c r="L164" s="11"/>
     </row>
-    <row r="165" spans="1:12" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A165" s="10">
         <v>164</v>
       </c>
@@ -7505,7 +7504,7 @@
       </c>
       <c r="L165" s="11"/>
     </row>
-    <row r="166" spans="1:12" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A166" s="10">
         <v>165</v>
       </c>
@@ -7542,16 +7541,7 @@
       <c r="L166" s="11"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L166" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="Action through Vanilla (Open UI desktop)/Guided Journey from Open UI Tablet"/>
-        <filter val="Guided Journey"/>
-        <filter val="Guided Journey in Open UI Tablet/Action Through Vanilla (Open UI Desktop)"/>
-        <filter val="Guided Journey/Action Through Vanilla (Open UI Desktop)"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:L166" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddFooter>&amp;L&amp;"Aptos"&amp;10 &amp;K000000_x000D_# Public</oddFooter>

</xml_diff>